<commit_message>
static-route-missing-threshold: insert SQL statements mostly done
</commit_message>
<xml_diff>
--- a/Splunk Alerts 2026-02-17(working-document).xlsx
+++ b/Splunk Alerts 2026-02-17(working-document).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rndc/Desktop/Work related/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6CDA25-3FEA-3148-A046-AD782365E3A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD78F253-C864-124C-B8EA-66349564BA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" tabRatio="794" activeTab="10" xr2:uid="{2DE4A338-4516-EF4B-97BB-8C0493E05CC2}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20480" tabRatio="794" activeTab="10" xr2:uid="{2DE4A338-4516-EF4B-97BB-8C0493E05CC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress List" sheetId="5" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7648" uniqueCount="1793">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7649" uniqueCount="1794">
   <si>
     <t>SPLUNK DECOMISSIONING</t>
   </si>
@@ -6865,12 +6865,6 @@
     <t>TO: Teppi.Waxman@RNDC-USA.COM, stanley.monis@rndc-usa.com, SeoFoo.Dang@RNDC-USA.COM, Vincent.Labasan@RNDC-USA.COM, Amorsolo.Angco@rndc-usa.com, Wallace.Moniz@RNDC-USA.COM, Reoben.Aquino@RNDC-USA.COM, ashlyn.javier@rndc-usa.com CC: wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM</t>
   </si>
   <si>
-    <t xml:space="preserve">These 3 groups of warehouses under this alert SELECT different columns and differ between each other, though connection string is identical
-(DFB - MAWM - Standard Orders Deselected During Waving and 
-IND - MAWM - Standard Orders Deselected During Waving) ; (
-PEN - MAWM - Standard Orders Deselected During Waving); and (all remaining enabled alerts) </t>
-  </si>
-  <si>
     <t xml:space="preserve"> | dbxquery query="SELECT DISTINCT O.org_id,
                 O.original_order_id,
                 O.order_type,
@@ -8779,6 +8773,13 @@
   </si>
   <si>
     <t>Turn on in WMS Tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">These 2 groups of warehouses under this alert SELECT different columns and differ between each other, though connection string is identical (
+PEN - MAWM - Standard Orders Deselected During Waving); and (all remaining enabled alerts) </t>
+  </si>
+  <si>
+    <t>For DEN warehouse , "Search String" option was checked as result to be returned .</t>
   </si>
 </sst>
 </file>
@@ -9537,7 +9538,7 @@
     <xf numFmtId="0" fontId="16" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="248">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10114,6 +10115,45 @@
     <xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -10138,45 +10178,6 @@
     <xf numFmtId="0" fontId="1" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -10191,6 +10192,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -10913,34 +10930,34 @@
   <sheetData>
     <row r="1" spans="2:13" ht="16" thickBot="1"/>
     <row r="2" spans="2:13" ht="15" customHeight="1">
-      <c r="B2" s="216" t="s">
+      <c r="B2" s="229" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="217"/>
-      <c r="D2" s="217"/>
-      <c r="E2" s="217"/>
-      <c r="F2" s="217"/>
-      <c r="G2" s="217"/>
-      <c r="H2" s="217"/>
-      <c r="I2" s="217"/>
-      <c r="J2" s="217"/>
-      <c r="K2" s="217"/>
-      <c r="L2" s="217"/>
-      <c r="M2" s="218"/>
+      <c r="C2" s="230"/>
+      <c r="D2" s="230"/>
+      <c r="E2" s="230"/>
+      <c r="F2" s="230"/>
+      <c r="G2" s="230"/>
+      <c r="H2" s="230"/>
+      <c r="I2" s="230"/>
+      <c r="J2" s="230"/>
+      <c r="K2" s="230"/>
+      <c r="L2" s="230"/>
+      <c r="M2" s="231"/>
     </row>
     <row r="3" spans="2:13" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B3" s="219"/>
-      <c r="C3" s="220"/>
-      <c r="D3" s="220"/>
-      <c r="E3" s="220"/>
-      <c r="F3" s="220"/>
-      <c r="G3" s="220"/>
-      <c r="H3" s="220"/>
-      <c r="I3" s="220"/>
-      <c r="J3" s="220"/>
-      <c r="K3" s="220"/>
-      <c r="L3" s="220"/>
-      <c r="M3" s="221"/>
+      <c r="B3" s="232"/>
+      <c r="C3" s="233"/>
+      <c r="D3" s="233"/>
+      <c r="E3" s="233"/>
+      <c r="F3" s="233"/>
+      <c r="G3" s="233"/>
+      <c r="H3" s="233"/>
+      <c r="I3" s="233"/>
+      <c r="J3" s="233"/>
+      <c r="K3" s="233"/>
+      <c r="L3" s="233"/>
+      <c r="M3" s="234"/>
     </row>
     <row r="4" spans="2:13" ht="17" thickBot="1">
       <c r="B4" s="182" t="s">
@@ -11261,32 +11278,32 @@
     </row>
     <row r="14" spans="2:13" ht="16" thickBot="1"/>
     <row r="15" spans="2:13" ht="15" customHeight="1">
-      <c r="B15" s="216" t="s">
+      <c r="B15" s="229" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="217"/>
-      <c r="D15" s="217"/>
-      <c r="E15" s="217"/>
-      <c r="F15" s="217"/>
-      <c r="G15" s="217"/>
-      <c r="H15" s="217"/>
-      <c r="I15" s="217"/>
-      <c r="J15" s="217"/>
-      <c r="K15" s="217"/>
-      <c r="L15" s="218"/>
+      <c r="C15" s="230"/>
+      <c r="D15" s="230"/>
+      <c r="E15" s="230"/>
+      <c r="F15" s="230"/>
+      <c r="G15" s="230"/>
+      <c r="H15" s="230"/>
+      <c r="I15" s="230"/>
+      <c r="J15" s="230"/>
+      <c r="K15" s="230"/>
+      <c r="L15" s="231"/>
     </row>
     <row r="16" spans="2:13" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B16" s="219"/>
-      <c r="C16" s="220"/>
-      <c r="D16" s="220"/>
-      <c r="E16" s="220"/>
-      <c r="F16" s="220"/>
-      <c r="G16" s="220"/>
-      <c r="H16" s="220"/>
-      <c r="I16" s="220"/>
-      <c r="J16" s="220"/>
-      <c r="K16" s="220"/>
-      <c r="L16" s="221"/>
+      <c r="B16" s="232"/>
+      <c r="C16" s="233"/>
+      <c r="D16" s="233"/>
+      <c r="E16" s="233"/>
+      <c r="F16" s="233"/>
+      <c r="G16" s="233"/>
+      <c r="H16" s="233"/>
+      <c r="I16" s="233"/>
+      <c r="J16" s="233"/>
+      <c r="K16" s="233"/>
+      <c r="L16" s="234"/>
     </row>
     <row r="17" spans="2:12" ht="33" thickBot="1">
       <c r="B17" s="84" t="s">
@@ -11298,24 +11315,24 @@
       <c r="D17" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="231" t="s">
+      <c r="E17" s="228" t="s">
         <v>28</v>
       </c>
-      <c r="F17" s="231"/>
+      <c r="F17" s="228"/>
       <c r="G17" s="85" t="s">
         <v>29</v>
       </c>
-      <c r="H17" s="234" t="s">
+      <c r="H17" s="227" t="s">
         <v>28</v>
       </c>
-      <c r="I17" s="234"/>
+      <c r="I17" s="227"/>
       <c r="J17" s="140" t="s">
         <v>30</v>
       </c>
-      <c r="K17" s="222" t="s">
+      <c r="K17" s="235" t="s">
         <v>28</v>
       </c>
-      <c r="L17" s="223"/>
+      <c r="L17" s="236"/>
     </row>
     <row r="18" spans="2:12" ht="63" customHeight="1">
       <c r="B18" s="86" t="s">
@@ -11327,24 +11344,24 @@
       <c r="D18" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="229" t="s">
+      <c r="E18" s="225" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="230"/>
+      <c r="F18" s="226"/>
       <c r="G18" s="88" t="s">
         <v>32</v>
       </c>
-      <c r="H18" s="229" t="s">
+      <c r="H18" s="225" t="s">
         <v>34</v>
       </c>
-      <c r="I18" s="230"/>
+      <c r="I18" s="226"/>
       <c r="J18" s="142" t="s">
         <v>35</v>
       </c>
-      <c r="K18" s="224" t="s">
+      <c r="K18" s="220" t="s">
         <v>36</v>
       </c>
-      <c r="L18" s="225"/>
+      <c r="L18" s="221"/>
     </row>
     <row r="19" spans="2:12">
       <c r="B19" s="81" t="s">
@@ -11356,22 +11373,22 @@
       <c r="D19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="228" t="s">
+      <c r="E19" s="222" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="225"/>
+      <c r="F19" s="221"/>
       <c r="G19" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="H19" s="228" t="s">
+      <c r="H19" s="222" t="s">
         <v>39</v>
       </c>
-      <c r="I19" s="225"/>
+      <c r="I19" s="221"/>
       <c r="J19" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K19" s="226"/>
-      <c r="L19" s="227"/>
+      <c r="K19" s="216"/>
+      <c r="L19" s="217"/>
     </row>
     <row r="20" spans="2:12" ht="30" customHeight="1">
       <c r="B20" s="81" t="s">
@@ -11383,22 +11400,22 @@
       <c r="D20" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="228" t="s">
+      <c r="E20" s="222" t="s">
         <v>42</v>
       </c>
-      <c r="F20" s="225"/>
+      <c r="F20" s="221"/>
       <c r="G20" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="H20" s="228" t="s">
+      <c r="H20" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="I20" s="225"/>
+      <c r="I20" s="221"/>
       <c r="J20" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K20" s="226"/>
-      <c r="L20" s="227"/>
+      <c r="K20" s="216"/>
+      <c r="L20" s="217"/>
     </row>
     <row r="21" spans="2:12" ht="36" customHeight="1">
       <c r="B21" s="81" t="s">
@@ -11410,22 +11427,22 @@
       <c r="D21" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="228" t="s">
+      <c r="E21" s="222" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="225"/>
+      <c r="F21" s="221"/>
       <c r="G21" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="H21" s="228" t="s">
+      <c r="H21" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="I21" s="225"/>
+      <c r="I21" s="221"/>
       <c r="J21" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K21" s="226"/>
-      <c r="L21" s="227"/>
+      <c r="K21" s="216"/>
+      <c r="L21" s="217"/>
     </row>
     <row r="22" spans="2:12" ht="29.25" customHeight="1">
       <c r="B22" s="81" t="s">
@@ -11437,22 +11454,22 @@
       <c r="D22" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="228" t="s">
+      <c r="E22" s="222" t="s">
         <v>42</v>
       </c>
-      <c r="F22" s="225"/>
+      <c r="F22" s="221"/>
       <c r="G22" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="H22" s="228" t="s">
+      <c r="H22" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="I22" s="225"/>
+      <c r="I22" s="221"/>
       <c r="J22" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K22" s="226"/>
-      <c r="L22" s="227"/>
+      <c r="K22" s="216"/>
+      <c r="L22" s="217"/>
     </row>
     <row r="23" spans="2:12" ht="48.75" customHeight="1">
       <c r="B23" s="81" t="s">
@@ -11464,24 +11481,24 @@
       <c r="D23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="228" t="s">
+      <c r="E23" s="222" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="225"/>
+      <c r="F23" s="221"/>
       <c r="G23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="H23" s="228" t="s">
+      <c r="H23" s="222" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="225"/>
+      <c r="I23" s="221"/>
       <c r="J23" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K23" s="224" t="s">
+      <c r="K23" s="220" t="s">
         <v>36</v>
       </c>
-      <c r="L23" s="225"/>
+      <c r="L23" s="221"/>
     </row>
     <row r="24" spans="2:12" ht="30" customHeight="1">
       <c r="B24" s="81" t="s">
@@ -11493,22 +11510,22 @@
       <c r="D24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="228" t="s">
+      <c r="E24" s="222" t="s">
         <v>42</v>
       </c>
-      <c r="F24" s="225"/>
+      <c r="F24" s="221"/>
       <c r="G24" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="H24" s="228" t="s">
+      <c r="H24" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="I24" s="225"/>
+      <c r="I24" s="221"/>
       <c r="J24" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K24" s="226"/>
-      <c r="L24" s="227"/>
+      <c r="K24" s="216"/>
+      <c r="L24" s="217"/>
     </row>
     <row r="25" spans="2:12" ht="49.5" customHeight="1">
       <c r="B25" s="81" t="s">
@@ -11520,22 +11537,22 @@
       <c r="D25" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E25" s="228" t="s">
+      <c r="E25" s="222" t="s">
         <v>50</v>
       </c>
-      <c r="F25" s="225"/>
+      <c r="F25" s="221"/>
       <c r="G25" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="H25" s="228" t="s">
+      <c r="H25" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="I25" s="225"/>
+      <c r="I25" s="221"/>
       <c r="J25" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K25" s="226"/>
-      <c r="L25" s="227"/>
+      <c r="K25" s="216"/>
+      <c r="L25" s="217"/>
     </row>
     <row r="26" spans="2:12" ht="33" customHeight="1">
       <c r="B26" s="81" t="s">
@@ -11547,22 +11564,22 @@
       <c r="D26" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E26" s="228" t="s">
+      <c r="E26" s="222" t="s">
         <v>52</v>
       </c>
-      <c r="F26" s="225"/>
+      <c r="F26" s="221"/>
       <c r="G26" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="H26" s="228" t="s">
+      <c r="H26" s="222" t="s">
         <v>43</v>
       </c>
-      <c r="I26" s="225"/>
+      <c r="I26" s="221"/>
       <c r="J26" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="K26" s="226"/>
-      <c r="L26" s="227"/>
+      <c r="K26" s="216"/>
+      <c r="L26" s="217"/>
     </row>
     <row r="27" spans="2:12" ht="16" thickBot="1">
       <c r="B27" s="82" t="s">
@@ -11574,33 +11591,36 @@
       <c r="D27" s="83" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="232" t="s">
+      <c r="E27" s="223" t="s">
         <v>54</v>
       </c>
-      <c r="F27" s="233"/>
+      <c r="F27" s="224"/>
       <c r="G27" s="90" t="s">
         <v>40</v>
       </c>
-      <c r="H27" s="232" t="s">
+      <c r="H27" s="223" t="s">
         <v>43</v>
       </c>
-      <c r="I27" s="233"/>
+      <c r="I27" s="224"/>
       <c r="J27" s="144" t="s">
         <v>40</v>
       </c>
-      <c r="K27" s="235"/>
-      <c r="L27" s="236"/>
+      <c r="K27" s="218"/>
+      <c r="L27" s="219"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="B15:L16"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="B2:M3"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E19:F19"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="E27:F27"/>
@@ -11617,17 +11637,14 @@
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B15:L16"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="B2:M3"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K24:L24"/>
   </mergeCells>
   <conditionalFormatting sqref="C18:D27 G18:G27 J18:J27">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
@@ -11682,7 +11699,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F42BD6B3-ABAD-41C6-A5CA-CB7783A0CB85}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:V109"/>
+  <dimension ref="A1:W109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -11705,7 +11722,7 @@
     <col min="22" max="22" width="8.83203125" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="32">
+    <row r="1" spans="1:23" ht="32">
       <c r="A1" t="s">
         <v>1528</v>
       </c>
@@ -11773,7 +11790,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="255" hidden="1" customHeight="1">
+    <row r="2" spans="1:23" ht="255" hidden="1" customHeight="1">
       <c r="A2">
         <v>7</v>
       </c>
@@ -11828,260 +11845,281 @@
         <v>1547</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="133.25" customHeight="1">
-      <c r="A3">
+    <row r="3" spans="1:23" ht="133.25" customHeight="1">
+      <c r="A3" s="213">
         <v>10</v>
       </c>
-      <c r="B3"/>
-      <c r="C3" s="125">
+      <c r="B3" s="213"/>
+      <c r="C3" s="246">
         <v>5</v>
       </c>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="214" t="s">
         <v>1540</v>
       </c>
-      <c r="E3" s="38" t="str">
+      <c r="E3" s="214" t="str">
         <f>'Final_List-Alerts'!A10</f>
         <v>ORDERS STUCK IN CREATED STATUS &gt; 15 MINUTES</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="F3" s="214" t="s">
         <v>1548</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="213" t="s">
         <v>1549</v>
       </c>
-      <c r="H3" s="38" t="s">
+      <c r="H3" s="214" t="s">
         <v>1183</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="213" t="s">
         <v>1550</v>
       </c>
-      <c r="J3" s="38" t="s">
+      <c r="J3" s="214" t="s">
         <v>1551</v>
       </c>
-      <c r="K3" s="38" t="s">
+      <c r="K3" s="214" t="s">
         <v>1543</v>
       </c>
-      <c r="L3" s="38" t="s">
+      <c r="L3" s="214" t="s">
         <v>1544</v>
       </c>
-      <c r="M3" s="38" t="s">
+      <c r="M3" s="214" t="s">
         <v>1552</v>
       </c>
-      <c r="N3" s="38" t="s">
+      <c r="N3" s="214" t="s">
         <v>1553</v>
       </c>
-      <c r="O3" s="38"/>
-      <c r="P3" s="196"/>
-      <c r="Q3" s="196"/>
-      <c r="R3" s="196"/>
-      <c r="S3" s="196">
+      <c r="O3" s="214"/>
+      <c r="P3" s="215"/>
+      <c r="Q3" s="215"/>
+      <c r="R3" s="215"/>
+      <c r="S3" s="215">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" ht="409.6">
-      <c r="A4">
+      <c r="T3" s="213"/>
+      <c r="U3" s="213"/>
+      <c r="V3" s="214"/>
+      <c r="W3" s="213"/>
+    </row>
+    <row r="4" spans="1:23" s="242" customFormat="1" ht="409.6">
+      <c r="A4" s="213">
         <v>11</v>
       </c>
-      <c r="B4"/>
-      <c r="C4" s="125">
+      <c r="B4" s="213"/>
+      <c r="C4" s="246">
         <v>6</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="214" t="s">
         <v>1540</v>
       </c>
-      <c r="E4" s="38" t="str">
+      <c r="E4" s="214" t="str">
         <f>'Final_List-Alerts'!A11</f>
         <v>STANDARD ORDERS DESELECTED DURING WAVING</v>
       </c>
-      <c r="F4" s="38" t="s">
+      <c r="F4" s="214" t="s">
         <v>1554</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="213" t="s">
         <v>1549</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="214" t="s">
         <v>1183</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="213" t="s">
         <v>1550</v>
       </c>
-      <c r="J4" s="38" t="s">
+      <c r="J4" s="214" t="s">
         <v>1555</v>
       </c>
-      <c r="K4" s="38" t="s">
+      <c r="K4" s="214" t="s">
         <v>1543</v>
       </c>
-      <c r="L4" s="38" t="s">
+      <c r="L4" s="214" t="s">
         <v>1544</v>
       </c>
-      <c r="M4" s="38" t="s">
+      <c r="M4" s="214" t="s">
         <v>1556</v>
       </c>
-      <c r="N4" s="38" t="s">
+      <c r="N4" s="214" t="s">
         <v>1557</v>
       </c>
-      <c r="O4" s="38"/>
-      <c r="P4" s="196"/>
-      <c r="Q4" s="196"/>
-      <c r="R4" s="196"/>
-      <c r="S4" s="196">
+      <c r="O4" s="214"/>
+      <c r="P4" s="215"/>
+      <c r="Q4" s="215"/>
+      <c r="R4" s="215"/>
+      <c r="S4" s="215">
         <v>1</v>
       </c>
-      <c r="V4" s="38" t="s">
-        <v>1558</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" ht="409.6">
-      <c r="A5">
+      <c r="T4" s="213"/>
+      <c r="U4" s="213"/>
+      <c r="V4" s="214" t="s">
+        <v>1792</v>
+      </c>
+      <c r="W4" s="213"/>
+    </row>
+    <row r="5" spans="1:23" ht="409.6">
+      <c r="A5" s="172">
         <v>12</v>
       </c>
-      <c r="B5"/>
-      <c r="C5" s="125">
+      <c r="B5" s="172"/>
+      <c r="C5" s="176">
         <v>7</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="173" t="s">
         <v>1540</v>
       </c>
-      <c r="E5" s="38" t="str">
+      <c r="E5" s="173" t="str">
         <f>'Final_List-Alerts'!A12</f>
         <v>STANDARD ORDERS W/ NO DESIGNATED OR ASSIGNED SHIPMENTS CREATED</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="F5" s="173" t="s">
+        <v>1558</v>
+      </c>
+      <c r="G5" s="172" t="s">
+        <v>1549</v>
+      </c>
+      <c r="H5" s="173" t="s">
+        <v>1183</v>
+      </c>
+      <c r="I5" s="172" t="s">
+        <v>1550</v>
+      </c>
+      <c r="J5" s="173" t="s">
         <v>1559</v>
       </c>
-      <c r="G5" t="s">
-        <v>1549</v>
-      </c>
-      <c r="H5" s="38" t="s">
-        <v>1183</v>
-      </c>
-      <c r="I5" t="s">
-        <v>1550</v>
-      </c>
-      <c r="J5" s="38" t="s">
+      <c r="K5" s="173" t="s">
+        <v>1543</v>
+      </c>
+      <c r="L5" s="173" t="s">
+        <v>1544</v>
+      </c>
+      <c r="M5" s="173" t="s">
         <v>1560</v>
       </c>
-      <c r="K5" s="38" t="s">
-        <v>1543</v>
-      </c>
-      <c r="L5" s="38" t="s">
-        <v>1544</v>
-      </c>
-      <c r="M5" s="38" t="s">
+      <c r="N5" s="173" t="s">
         <v>1561</v>
       </c>
-      <c r="N5" s="38" t="s">
-        <v>1562</v>
-      </c>
-      <c r="O5" s="38"/>
-      <c r="P5" s="196"/>
-      <c r="Q5" s="196"/>
-      <c r="R5" s="196"/>
-      <c r="S5" s="196">
+      <c r="O5" s="173"/>
+      <c r="P5" s="247"/>
+      <c r="Q5" s="247"/>
+      <c r="R5" s="247"/>
+      <c r="S5" s="247">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" ht="409.6">
-      <c r="A6">
+      <c r="T5" s="172"/>
+      <c r="U5" s="172"/>
+      <c r="V5" s="173"/>
+      <c r="W5" s="172"/>
+    </row>
+    <row r="6" spans="1:23" ht="409.6">
+      <c r="A6" s="172">
         <v>15</v>
       </c>
-      <c r="B6"/>
-      <c r="C6" s="125">
+      <c r="B6" s="172"/>
+      <c r="C6" s="176">
         <v>8</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="173" t="s">
         <v>1540</v>
       </c>
-      <c r="E6" s="38" t="str">
+      <c r="E6" s="173" t="str">
         <f>'Final_List-Alerts'!A15</f>
         <v>STANDARD ORDERS W/ NO DESIGNATED SHIPMENTS CREATED</v>
       </c>
-      <c r="F6" s="38" t="s">
+      <c r="F6" s="173" t="s">
+        <v>1562</v>
+      </c>
+      <c r="G6" s="172" t="s">
+        <v>1549</v>
+      </c>
+      <c r="H6" s="173" t="s">
+        <v>1183</v>
+      </c>
+      <c r="I6" s="172" t="s">
+        <v>1550</v>
+      </c>
+      <c r="J6" s="173" t="s">
         <v>1563</v>
       </c>
-      <c r="G6" t="s">
-        <v>1549</v>
-      </c>
-      <c r="H6" s="38" t="s">
-        <v>1183</v>
-      </c>
-      <c r="I6" t="s">
-        <v>1550</v>
-      </c>
-      <c r="J6" s="38" t="s">
+      <c r="K6" s="173" t="s">
+        <v>1543</v>
+      </c>
+      <c r="L6" s="173" t="s">
+        <v>1544</v>
+      </c>
+      <c r="M6" s="173" t="s">
         <v>1564</v>
       </c>
-      <c r="K6" s="38" t="s">
-        <v>1543</v>
-      </c>
-      <c r="L6" s="38" t="s">
-        <v>1544</v>
-      </c>
-      <c r="M6" s="38" t="s">
+      <c r="N6" s="173" t="s">
         <v>1565</v>
       </c>
-      <c r="N6" s="38" t="s">
-        <v>1566</v>
-      </c>
-      <c r="O6" s="38"/>
-      <c r="P6" s="196"/>
-      <c r="Q6" s="196"/>
-      <c r="R6" s="196"/>
-      <c r="S6" s="196">
+      <c r="O6" s="173"/>
+      <c r="P6" s="247"/>
+      <c r="Q6" s="247"/>
+      <c r="R6" s="247"/>
+      <c r="S6" s="247">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" ht="128">
-      <c r="A7">
+      <c r="T6" s="172"/>
+      <c r="U6" s="172"/>
+      <c r="V6" s="173" t="s">
+        <v>1793</v>
+      </c>
+      <c r="W6" s="172"/>
+    </row>
+    <row r="7" spans="1:23" ht="128">
+      <c r="A7" s="242">
         <v>17</v>
       </c>
-      <c r="B7"/>
-      <c r="C7" s="125">
+      <c r="B7" s="242"/>
+      <c r="C7" s="243">
         <v>9</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="244" t="s">
         <v>1540</v>
       </c>
-      <c r="E7" s="38" t="str">
+      <c r="E7" s="244" t="str">
         <f>'Final_List-Alerts'!A17</f>
         <v>STATIC ROUTE MISSING THRESHOLD VALUE</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="F7" s="244" t="s">
+        <v>1566</v>
+      </c>
+      <c r="G7" s="242" t="s">
+        <v>1549</v>
+      </c>
+      <c r="H7" s="244" t="s">
+        <v>1183</v>
+      </c>
+      <c r="I7" s="242" t="s">
+        <v>1550</v>
+      </c>
+      <c r="J7" s="244" t="s">
         <v>1567</v>
       </c>
-      <c r="G7" t="s">
-        <v>1549</v>
-      </c>
-      <c r="H7" s="38" t="s">
-        <v>1183</v>
-      </c>
-      <c r="I7" t="s">
-        <v>1550</v>
-      </c>
-      <c r="J7" s="38" t="s">
+      <c r="K7" s="244" t="s">
+        <v>1543</v>
+      </c>
+      <c r="L7" s="244" t="s">
+        <v>1544</v>
+      </c>
+      <c r="M7" s="244" t="s">
         <v>1568</v>
       </c>
-      <c r="K7" s="38" t="s">
-        <v>1543</v>
-      </c>
-      <c r="L7" s="38" t="s">
-        <v>1544</v>
-      </c>
-      <c r="M7" s="38" t="s">
+      <c r="N7" s="244" t="s">
         <v>1569</v>
       </c>
-      <c r="N7" s="38" t="s">
-        <v>1570</v>
-      </c>
-      <c r="O7" s="38"/>
-      <c r="P7" s="196"/>
-      <c r="Q7" s="196"/>
-      <c r="R7" s="196"/>
-      <c r="S7" s="196">
+      <c r="O7" s="244"/>
+      <c r="P7" s="245"/>
+      <c r="Q7" s="245"/>
+      <c r="R7" s="245"/>
+      <c r="S7" s="245">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" ht="240">
+      <c r="T7" s="242"/>
+      <c r="U7" s="242"/>
+      <c r="V7" s="244"/>
+      <c r="W7" s="242"/>
+    </row>
+    <row r="8" spans="1:23" ht="240">
       <c r="A8">
         <v>20</v>
       </c>
@@ -12097,7 +12135,7 @@
         <v>STATIC ROUTE UI MISSING DFLT VALUE</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="G8" t="s">
         <v>1549</v>
@@ -12109,7 +12147,7 @@
         <v>1550</v>
       </c>
       <c r="J8" s="38" t="s">
-        <v>1572</v>
+        <v>1571</v>
       </c>
       <c r="K8" s="38" t="s">
         <v>1543</v>
@@ -12118,10 +12156,10 @@
         <v>1544</v>
       </c>
       <c r="M8" s="38" t="s">
+        <v>1572</v>
+      </c>
+      <c r="N8" s="38" t="s">
         <v>1573</v>
-      </c>
-      <c r="N8" s="38" t="s">
-        <v>1574</v>
       </c>
       <c r="O8" s="38"/>
       <c r="P8" s="196"/>
@@ -12131,7 +12169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="409.6">
+    <row r="9" spans="1:23" ht="409.6">
       <c r="A9">
         <v>21</v>
       </c>
@@ -12147,7 +12185,7 @@
         <v>ROUTES WITH MULTIPLE WAVE NUMBERS</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>1575</v>
+        <v>1574</v>
       </c>
       <c r="G9" t="s">
         <v>1549</v>
@@ -12159,19 +12197,19 @@
         <v>1550</v>
       </c>
       <c r="J9" s="38" t="s">
+        <v>1575</v>
+      </c>
+      <c r="K9" s="38" t="s">
         <v>1576</v>
-      </c>
-      <c r="K9" s="38" t="s">
-        <v>1577</v>
       </c>
       <c r="L9" s="38" t="s">
         <v>1544</v>
       </c>
       <c r="M9" s="38" t="s">
+        <v>1577</v>
+      </c>
+      <c r="N9" s="38" t="s">
         <v>1578</v>
-      </c>
-      <c r="N9" s="38" t="s">
-        <v>1579</v>
       </c>
       <c r="O9" s="38"/>
       <c r="P9" s="196"/>
@@ -12181,10 +12219,10 @@
         <v>1</v>
       </c>
       <c r="V9" s="38" t="s">
-        <v>1580</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="32" hidden="1" customHeight="1">
+        <v>1579</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="32" hidden="1" customHeight="1">
       <c r="A10">
         <v>22</v>
       </c>
@@ -12197,7 +12235,7 @@
         <v>Item Loc Prod (ITEMLOC_PRD)</v>
       </c>
       <c r="F10" s="41" t="s">
-        <v>1581</v>
+        <v>1580</v>
       </c>
       <c r="G10" s="41"/>
       <c r="H10" s="41"/>
@@ -12215,7 +12253,7 @@
       <c r="U10" s="41"/>
       <c r="V10" s="41"/>
     </row>
-    <row r="11" spans="1:22" ht="160" hidden="1">
+    <row r="11" spans="1:23" ht="160" hidden="1">
       <c r="A11">
         <v>24</v>
       </c>
@@ -12233,22 +12271,22 @@
         <v>DUPLICATE PIX S IN MIDDLEWARE WMS</v>
       </c>
       <c r="F11" s="38" t="s">
+        <v>1581</v>
+      </c>
+      <c r="G11" t="s">
         <v>1582</v>
-      </c>
-      <c r="G11" t="s">
-        <v>1583</v>
       </c>
       <c r="H11" s="38" t="s">
         <v>171</v>
       </c>
       <c r="I11" t="s">
+        <v>1583</v>
+      </c>
+      <c r="J11" s="38" t="s">
         <v>1584</v>
       </c>
-      <c r="J11" s="38" t="s">
-        <v>1585</v>
-      </c>
       <c r="K11" s="38" t="s">
-        <v>1577</v>
+        <v>1576</v>
       </c>
       <c r="L11" s="38" t="s">
         <v>1544</v>
@@ -12257,7 +12295,7 @@
         <v>1556</v>
       </c>
       <c r="N11" s="38" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="O11" s="38"/>
       <c r="P11" s="196"/>
@@ -12267,7 +12305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="288" hidden="1">
+    <row r="12" spans="1:23" ht="288" hidden="1">
       <c r="A12">
         <v>25</v>
       </c>
@@ -12283,7 +12321,7 @@
         <v>DUPLICATE SHIP CONFIRM</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>1586</v>
+        <v>1585</v>
       </c>
       <c r="G12" t="s">
         <v>214</v>
@@ -12295,7 +12333,7 @@
         <v>1541</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>1587</v>
+        <v>1586</v>
       </c>
       <c r="K12" s="38" t="s">
         <v>1543</v>
@@ -12307,7 +12345,7 @@
         <v>1556</v>
       </c>
       <c r="N12" s="38" t="s">
-        <v>1588</v>
+        <v>1587</v>
       </c>
       <c r="O12" s="38"/>
       <c r="P12" s="196"/>
@@ -12317,10 +12355,10 @@
         <v>1</v>
       </c>
       <c r="V12" s="38" t="s">
-        <v>1589</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" ht="365">
+        <v>1588</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" ht="365">
       <c r="A13">
         <v>27</v>
       </c>
@@ -12336,7 +12374,7 @@
         <v>INVENTORY ADJUSTMENT PIX MISSING REASON CODE</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>1590</v>
+        <v>1589</v>
       </c>
       <c r="G13" t="s">
         <v>1549</v>
@@ -12348,7 +12386,7 @@
         <v>1550</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>1591</v>
+        <v>1590</v>
       </c>
       <c r="K13" s="38" t="s">
         <v>1543</v>
@@ -12360,7 +12398,7 @@
         <v>1556</v>
       </c>
       <c r="N13" s="38" t="s">
-        <v>1592</v>
+        <v>1591</v>
       </c>
       <c r="O13" s="38"/>
       <c r="P13" s="196"/>
@@ -12370,10 +12408,10 @@
         <v>1</v>
       </c>
       <c r="V13" s="38" t="s">
-        <v>1593</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" ht="409.6">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" ht="409.6">
       <c r="A14">
         <v>28</v>
       </c>
@@ -12389,7 +12427,7 @@
         <v>ITEM LEVEL RECEIPTS WITH 0 QUANTITY</v>
       </c>
       <c r="F14" s="38" t="s">
-        <v>1594</v>
+        <v>1593</v>
       </c>
       <c r="G14" t="s">
         <v>1549</v>
@@ -12401,7 +12439,7 @@
         <v>1550</v>
       </c>
       <c r="J14" s="38" t="s">
-        <v>1595</v>
+        <v>1594</v>
       </c>
       <c r="K14" s="38" t="s">
         <v>1543</v>
@@ -12413,7 +12451,7 @@
         <v>116</v>
       </c>
       <c r="N14" s="38" t="s">
-        <v>1596</v>
+        <v>1595</v>
       </c>
       <c r="O14" s="38"/>
       <c r="P14" s="196"/>
@@ -12423,10 +12461,10 @@
         <v>1</v>
       </c>
       <c r="V14" s="38" t="s">
-        <v>1597</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" ht="409.6">
+        <v>1596</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="409.6">
       <c r="A15">
         <v>33</v>
       </c>
@@ -12442,7 +12480,7 @@
         <v>LONG RUNNING OR ABORTED WAVES</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>1598</v>
+        <v>1597</v>
       </c>
       <c r="G15" t="s">
         <v>1549</v>
@@ -12454,7 +12492,7 @@
         <v>1550</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>1599</v>
+        <v>1598</v>
       </c>
       <c r="K15" s="38" t="s">
         <v>1543</v>
@@ -12466,7 +12504,7 @@
         <v>177</v>
       </c>
       <c r="N15" s="38" t="s">
-        <v>1600</v>
+        <v>1599</v>
       </c>
       <c r="O15" s="38"/>
       <c r="P15" s="196"/>
@@ -12476,10 +12514,10 @@
         <v>1</v>
       </c>
       <c r="V15" s="38" t="s">
-        <v>1601</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22" ht="409.6" hidden="1">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" ht="409.6" hidden="1">
       <c r="A16">
         <v>34</v>
       </c>
@@ -12495,7 +12533,7 @@
         <v>MISSING ITEM LEVEL VERIFICATION PIX</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
       <c r="G16" t="s">
         <v>214</v>
@@ -12507,7 +12545,7 @@
         <v>1541</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>1603</v>
+        <v>1602</v>
       </c>
       <c r="K16" s="38" t="s">
         <v>1543</v>
@@ -12516,10 +12554,10 @@
         <v>1544</v>
       </c>
       <c r="M16" s="38" t="s">
-        <v>1604</v>
+        <v>1603</v>
       </c>
       <c r="N16" s="38" t="s">
-        <v>1588</v>
+        <v>1587</v>
       </c>
       <c r="O16" s="38"/>
       <c r="P16" s="196"/>
@@ -12529,7 +12567,7 @@
         <v>1</v>
       </c>
       <c r="V16" s="38" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="409.6">
@@ -12548,7 +12586,7 @@
         <v>ROUTED ORDERS CANCELLED</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="G17" t="s">
         <v>1549</v>
@@ -12560,7 +12598,7 @@
         <v>1550</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="K17" s="38" t="s">
         <v>1543</v>
@@ -12572,7 +12610,7 @@
         <v>1556</v>
       </c>
       <c r="N17" s="38" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="O17" s="38"/>
       <c r="P17" s="196"/>
@@ -12582,7 +12620,7 @@
         <v>1</v>
       </c>
       <c r="V17" s="38" t="s">
-        <v>1609</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="320">
@@ -12601,10 +12639,10 @@
         <v>ALL - MAWM - PIX Specification Found &gt; 1 Hour</v>
       </c>
       <c r="F18" s="38" t="s">
+        <v>1609</v>
+      </c>
+      <c r="G18" t="s">
         <v>1610</v>
-      </c>
-      <c r="G18" t="s">
-        <v>1611</v>
       </c>
       <c r="H18" s="38" t="s">
         <v>1183</v>
@@ -12613,19 +12651,19 @@
         <v>1550</v>
       </c>
       <c r="J18" s="38" t="s">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="K18" s="38" t="s">
-        <v>1577</v>
+        <v>1576</v>
       </c>
       <c r="L18" s="38" t="s">
         <v>1544</v>
       </c>
       <c r="M18" s="38" t="s">
+        <v>1612</v>
+      </c>
+      <c r="N18" s="38" t="s">
         <v>1613</v>
-      </c>
-      <c r="N18" s="38" t="s">
-        <v>1614</v>
       </c>
       <c r="O18" s="38"/>
     </row>
@@ -12645,7 +12683,7 @@
         <v>ALL - MAWM - Unprocessed or Failed Ship Confirms Last 24 Hours</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>1615</v>
+        <v>1614</v>
       </c>
       <c r="G19" s="38" t="s">
         <v>1549</v>
@@ -12660,16 +12698,16 @@
         <v>159</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L19" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M19" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N19" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O19" s="38"/>
       <c r="P19" s="196"/>
@@ -12695,10 +12733,10 @@
         <v>MATM - SPO Import Failure</v>
       </c>
       <c r="F20" s="38" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="G20" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="H20" s="38" t="s">
         <v>1183</v>
@@ -12707,19 +12745,19 @@
         <v>1550</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>1618</v>
+        <v>1617</v>
       </c>
       <c r="K20" s="38" t="s">
-        <v>1577</v>
+        <v>1576</v>
       </c>
       <c r="L20" s="38" t="s">
         <v>1544</v>
       </c>
       <c r="M20" s="38" t="s">
+        <v>1618</v>
+      </c>
+      <c r="N20" s="38" t="s">
         <v>1619</v>
-      </c>
-      <c r="N20" s="38" t="s">
-        <v>1620</v>
       </c>
       <c r="S20" s="196">
         <v>1</v>
@@ -12741,7 +12779,7 @@
         <v>SHIPPED OLPN W/ CONSOLIDATION LOCATION ASSIGNMENT</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>1621</v>
+        <v>1620</v>
       </c>
       <c r="G21" t="s">
         <v>1549</v>
@@ -12753,19 +12791,19 @@
         <v>1550</v>
       </c>
       <c r="J21" s="38" t="s">
-        <v>1622</v>
+        <v>1621</v>
       </c>
       <c r="K21" s="38" t="s">
-        <v>1577</v>
+        <v>1576</v>
       </c>
       <c r="L21" s="38" t="s">
         <v>1544</v>
       </c>
       <c r="M21" s="38" t="s">
+        <v>1622</v>
+      </c>
+      <c r="N21" s="38" t="s">
         <v>1623</v>
-      </c>
-      <c r="N21" s="38" t="s">
-        <v>1624</v>
       </c>
       <c r="O21" s="38"/>
       <c r="P21" s="196"/>
@@ -12775,7 +12813,7 @@
         <v>1</v>
       </c>
       <c r="V21" s="38" t="s">
-        <v>1625</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="22" spans="1:22" s="204" customFormat="1" ht="409.6">
@@ -12794,7 +12832,7 @@
         <v>TEMPORARY RESERVE LOCATIONS W/ ASSIGNMENTS, BUT NO INVENTORY</v>
       </c>
       <c r="F22" s="38" t="s">
-        <v>1626</v>
+        <v>1625</v>
       </c>
       <c r="G22" t="s">
         <v>1549</v>
@@ -12806,7 +12844,7 @@
         <v>1550</v>
       </c>
       <c r="J22" s="38" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="K22" s="38" t="s">
         <v>1543</v>
@@ -12815,10 +12853,10 @@
         <v>1544</v>
       </c>
       <c r="M22" s="38" t="s">
+        <v>1627</v>
+      </c>
+      <c r="N22" s="38" t="s">
         <v>1628</v>
-      </c>
-      <c r="N22" s="38" t="s">
-        <v>1629</v>
       </c>
       <c r="O22" s="38"/>
       <c r="P22" s="196"/>
@@ -12846,7 +12884,7 @@
         <v>TEMPORARY RESERVE LOCATIONS W/ INVENTORY, BUT NO ASSIGNMENTS</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="G23" t="s">
         <v>1549</v>
@@ -12867,10 +12905,10 @@
         <v>1544</v>
       </c>
       <c r="M23" s="38" t="s">
+        <v>1630</v>
+      </c>
+      <c r="N23" s="38" t="s">
         <v>1631</v>
-      </c>
-      <c r="N23" s="38" t="s">
-        <v>1632</v>
       </c>
       <c r="O23" s="38"/>
       <c r="P23" s="196"/>
@@ -12896,7 +12934,7 @@
         <v>POR - MAWM - Duplicate PIX's in Middleware WMS</v>
       </c>
       <c r="F24" s="38" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="G24" t="s">
         <v>1549</v>
@@ -12943,7 +12981,7 @@
         <v>ALL - MAWM - Inventory Adjustment PIX w/ Null PO Line</v>
       </c>
       <c r="F25" s="205" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="G25" s="204" t="s">
         <v>214</v>
@@ -12955,7 +12993,7 @@
         <v>1541</v>
       </c>
       <c r="J25" s="205" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="K25" s="205" t="s">
         <v>1543</v>
@@ -12964,10 +13002,10 @@
         <v>1544</v>
       </c>
       <c r="M25" s="205" t="s">
+        <v>1635</v>
+      </c>
+      <c r="N25" s="205" t="s">
         <v>1636</v>
-      </c>
-      <c r="N25" s="205" t="s">
-        <v>1637</v>
       </c>
       <c r="O25" s="205"/>
       <c r="P25" s="206">
@@ -12980,7 +13018,7 @@
       </c>
       <c r="U25" s="204"/>
       <c r="V25" s="205" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="272">
@@ -12999,7 +13037,7 @@
         <v>ALL - MAWM - In Packing oLPNS &gt; 5 Minutes</v>
       </c>
       <c r="F26" s="38" t="s">
-        <v>1639</v>
+        <v>1638</v>
       </c>
       <c r="G26" s="38" t="s">
         <v>1549</v>
@@ -13011,19 +13049,19 @@
         <v>1550</v>
       </c>
       <c r="J26" s="38" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="K26" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L26" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M26" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N26" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O26" s="38"/>
       <c r="P26" s="196"/>
@@ -13061,19 +13099,19 @@
         <v>1550</v>
       </c>
       <c r="J27" s="38" t="s">
-        <v>1641</v>
+        <v>1640</v>
       </c>
       <c r="K27" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L27" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M27" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N27" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O27" s="38"/>
       <c r="S27" s="196">
@@ -13096,7 +13134,7 @@
         <v>ALL - MAWM - Putaway Task is Open but iLPN is Putaway</v>
       </c>
       <c r="F28" s="38" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="G28" s="38" t="s">
         <v>1549</v>
@@ -13111,16 +13149,16 @@
         <v>224</v>
       </c>
       <c r="K28" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L28" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M28" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N28" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O28" s="38"/>
       <c r="P28" s="196"/>
@@ -13146,7 +13184,7 @@
         <v>ALL - MAWM - Task Completed or Cancelled w/ Open Task Details</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>1643</v>
+        <v>1642</v>
       </c>
       <c r="G29" s="38" t="s">
         <v>1549</v>
@@ -13158,19 +13196,19 @@
         <v>1550</v>
       </c>
       <c r="J29" s="38" t="s">
-        <v>1644</v>
+        <v>1643</v>
       </c>
       <c r="K29" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L29" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M29" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N29" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O29" s="38"/>
       <c r="P29" s="196"/>
@@ -13196,7 +13234,7 @@
         <v>ALL - MAWM - Task Open w/ Completed or Cancelled Task Details</v>
       </c>
       <c r="F30" s="38" t="s">
-        <v>1645</v>
+        <v>1644</v>
       </c>
       <c r="G30" s="38" t="s">
         <v>1549</v>
@@ -13211,16 +13249,16 @@
         <v>226</v>
       </c>
       <c r="K30" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L30" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M30" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N30" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O30" s="38"/>
       <c r="P30" s="196"/>
@@ -13246,7 +13284,7 @@
         <v>ALL - MAWM - Task ‘In Progress’ w/ Completed or Cancelled Task Details</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>1646</v>
+        <v>1645</v>
       </c>
       <c r="G31" s="38" t="s">
         <v>1549</v>
@@ -13261,16 +13299,16 @@
         <v>227</v>
       </c>
       <c r="K31" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L31" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M31" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N31" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="O31" s="38"/>
       <c r="P31" s="196"/>
@@ -13295,7 +13333,7 @@
         <v>ABQ - MAWM - Travel &gt; 4 Mins</v>
       </c>
       <c r="F32" s="38" t="s">
-        <v>1647</v>
+        <v>1646</v>
       </c>
       <c r="G32" s="38" t="s">
         <v>214</v>
@@ -13316,10 +13354,10 @@
         <v>1544</v>
       </c>
       <c r="M32" s="38" t="s">
+        <v>1647</v>
+      </c>
+      <c r="N32" s="38" t="s">
         <v>1648</v>
-      </c>
-      <c r="N32" s="38" t="s">
-        <v>1649</v>
       </c>
       <c r="S32">
         <v>1</v>
@@ -13340,19 +13378,19 @@
         <v>ASN S WITH NO ASN LEVEL VERIFICATION &gt; 5DAYS</v>
       </c>
       <c r="F33" s="38" t="s">
+        <v>1649</v>
+      </c>
+      <c r="G33" s="38" t="s">
         <v>1650</v>
       </c>
-      <c r="G33" s="38" t="s">
+      <c r="H33" s="38" t="s">
+        <v>1615</v>
+      </c>
+      <c r="I33" s="38" t="s">
+        <v>1615</v>
+      </c>
+      <c r="J33" t="s">
         <v>1651</v>
-      </c>
-      <c r="H33" s="38" t="s">
-        <v>1616</v>
-      </c>
-      <c r="I33" s="38" t="s">
-        <v>1616</v>
-      </c>
-      <c r="J33" t="s">
-        <v>1652</v>
       </c>
       <c r="K33" s="38" t="s">
         <v>1543</v>
@@ -13361,13 +13399,13 @@
         <v>1544</v>
       </c>
       <c r="M33" s="38" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="S33" s="196">
         <v>1</v>
       </c>
       <c r="V33" s="38" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="34" spans="1:22" ht="409.6">
@@ -13385,7 +13423,7 @@
         <v>ILPNS WITH MISSING PHYSICALENTITYCODEID</v>
       </c>
       <c r="F34" s="38" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="G34" s="38" t="s">
         <v>1549</v>
@@ -13397,7 +13435,7 @@
         <v>1550</v>
       </c>
       <c r="J34" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="K34" s="38" t="s">
         <v>1543</v>
@@ -13406,10 +13444,10 @@
         <v>1544</v>
       </c>
       <c r="M34" s="38" t="s">
+        <v>1656</v>
+      </c>
+      <c r="N34" s="38" t="s">
         <v>1657</v>
-      </c>
-      <c r="N34" s="38" t="s">
-        <v>1658</v>
       </c>
       <c r="S34" s="196">
         <v>1</v>
@@ -13431,7 +13469,7 @@
         <v>LIA RECORDS WITH PACK UOM TYPE POPULATED</v>
       </c>
       <c r="F35" s="214" t="s">
-        <v>1659</v>
+        <v>1658</v>
       </c>
       <c r="G35" s="214" t="s">
         <v>1549</v>
@@ -13443,7 +13481,7 @@
         <v>1550</v>
       </c>
       <c r="J35" s="213" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="K35" s="214" t="s">
         <v>1543</v>
@@ -13455,7 +13493,7 @@
         <v>1556</v>
       </c>
       <c r="N35" s="214" t="s">
-        <v>1661</v>
+        <v>1660</v>
       </c>
       <c r="S35" s="215">
         <v>1</v>
@@ -13477,7 +13515,7 @@
         <v>LOCATION POSITION &gt; STREET LENGTH</v>
       </c>
       <c r="F36" s="38" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="G36" s="38" t="s">
         <v>214</v>
@@ -13489,7 +13527,7 @@
         <v>1550</v>
       </c>
       <c r="J36" t="s">
-        <v>1663</v>
+        <v>1662</v>
       </c>
       <c r="K36" s="38" t="s">
         <v>1543</v>
@@ -13498,16 +13536,16 @@
         <v>1544</v>
       </c>
       <c r="M36" s="38" t="s">
-        <v>1664</v>
+        <v>1663</v>
       </c>
       <c r="N36" s="38" t="s">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="S36" s="196">
         <v>1</v>
       </c>
       <c r="V36" s="38" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="37" spans="1:22" ht="409.6">
@@ -13525,7 +13563,7 @@
         <v>LOCATIONS W/ INVENTORY FOR ITEMS NOT ASSIGNED</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>1666</v>
+        <v>1665</v>
       </c>
       <c r="G37" s="38" t="s">
         <v>1549</v>
@@ -13537,7 +13575,7 @@
         <v>1550</v>
       </c>
       <c r="J37" s="38" t="s">
-        <v>1667</v>
+        <v>1666</v>
       </c>
       <c r="K37" s="38" t="s">
         <v>1543</v>
@@ -13549,13 +13587,13 @@
         <v>1556</v>
       </c>
       <c r="N37" s="38" t="s">
-        <v>1668</v>
+        <v>1667</v>
       </c>
       <c r="S37" s="196">
         <v>1</v>
       </c>
       <c r="V37" s="38" t="s">
-        <v>1669</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="38" spans="1:22" ht="128" hidden="1">
@@ -13563,7 +13601,7 @@
         <v>53</v>
       </c>
       <c r="B38" s="41" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="C38" s="38" t="s">
         <v>69</v>
@@ -13576,22 +13614,22 @@
         <v>SPLUNK API SCRIPTS SUMMARY</v>
       </c>
       <c r="F38" s="38" t="s">
-        <v>1671</v>
+        <v>1670</v>
       </c>
       <c r="G38" s="38" t="s">
         <v>184</v>
       </c>
       <c r="H38" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="I38" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="J38" s="38" t="s">
+        <v>1671</v>
+      </c>
+      <c r="K38" s="38" t="s">
         <v>1672</v>
-      </c>
-      <c r="K38" s="38" t="s">
-        <v>1673</v>
       </c>
       <c r="L38" s="38" t="s">
         <v>1544</v>
@@ -13600,13 +13638,13 @@
         <v>1556</v>
       </c>
       <c r="N38" s="38" t="s">
-        <v>1674</v>
+        <v>1673</v>
       </c>
       <c r="O38">
         <v>1</v>
       </c>
       <c r="V38" s="38" t="s">
-        <v>1675</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="39" spans="1:22" ht="224">
@@ -13624,7 +13662,7 @@
         <v>USERS W/ INCORRECT USER DEFAULT CONFIGURATION</v>
       </c>
       <c r="F39" s="38" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="G39" s="38" t="s">
         <v>1549</v>
@@ -13636,7 +13674,7 @@
         <v>1550</v>
       </c>
       <c r="J39" s="38" t="s">
-        <v>1677</v>
+        <v>1676</v>
       </c>
       <c r="K39" s="38" t="s">
         <v>1543</v>
@@ -13645,10 +13683,10 @@
         <v>1544</v>
       </c>
       <c r="M39" s="38" t="s">
+        <v>1677</v>
+      </c>
+      <c r="N39" s="38" t="s">
         <v>1678</v>
-      </c>
-      <c r="N39" s="38" t="s">
-        <v>1679</v>
       </c>
       <c r="S39" s="196">
         <v>1</v>
@@ -13681,7 +13719,7 @@
         <v>1550</v>
       </c>
       <c r="J40" s="38" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="K40" s="38" t="s">
         <v>1543</v>
@@ -13690,10 +13728,10 @@
         <v>1544</v>
       </c>
       <c r="M40" s="38" t="s">
+        <v>1680</v>
+      </c>
+      <c r="N40" s="38" t="s">
         <v>1681</v>
-      </c>
-      <c r="N40" s="38" t="s">
-        <v>1682</v>
       </c>
       <c r="S40" s="196">
         <v>1</v>
@@ -13714,7 +13752,7 @@
         <v>ALL - MAWM - Pallet LPNs w/ Inventory Records</v>
       </c>
       <c r="F41" s="38" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="G41" s="38" t="s">
         <v>1549</v>
@@ -13729,16 +13767,16 @@
         <v>189</v>
       </c>
       <c r="K41" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L41" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M41" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N41" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="S41" s="196">
         <v>1</v>
@@ -13759,7 +13797,7 @@
         <v>ALL - MAWM - oLPNs w/ Multiple Details of the Same Item</v>
       </c>
       <c r="F42" s="38" t="s">
-        <v>1684</v>
+        <v>1683</v>
       </c>
       <c r="G42" s="38" t="s">
         <v>1549</v>
@@ -13774,16 +13812,16 @@
         <v>192</v>
       </c>
       <c r="K42" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L42" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M42" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N42" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="S42" s="196">
         <v>1</v>
@@ -13804,7 +13842,7 @@
         <v>OPEN ORDER IN WM &gt; 1 WEEK</v>
       </c>
       <c r="F43" s="38" t="s">
-        <v>1685</v>
+        <v>1684</v>
       </c>
       <c r="G43" s="38" t="s">
         <v>1549</v>
@@ -13816,19 +13854,19 @@
         <v>1550</v>
       </c>
       <c r="J43" s="38" t="s">
-        <v>1686</v>
+        <v>1685</v>
       </c>
       <c r="K43" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L43" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M43" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N43" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="S43" s="196">
         <v>1</v>
@@ -13849,7 +13887,7 @@
         <v>All - MAWM - Multiple Order Lines Per Original Order Line</v>
       </c>
       <c r="F44" s="38" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G44" s="38" t="s">
         <v>1549</v>
@@ -13861,19 +13899,19 @@
         <v>1550</v>
       </c>
       <c r="J44" s="38" t="s">
-        <v>1688</v>
+        <v>1687</v>
       </c>
       <c r="K44" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L44" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M44" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N44" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="S44" s="196">
         <v>1</v>
@@ -13894,7 +13932,7 @@
         <v>ALL - MAWM - Items Weight with Large Dimensions</v>
       </c>
       <c r="F45" s="38" t="s">
-        <v>1689</v>
+        <v>1688</v>
       </c>
       <c r="G45" s="38" t="s">
         <v>1549</v>
@@ -13906,19 +13944,19 @@
         <v>1550</v>
       </c>
       <c r="J45" s="38" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
       <c r="K45" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L45" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M45" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N45" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="S45" s="196">
         <v>1</v>
@@ -13936,7 +13974,7 @@
         <v>ALL - MAWM - Items Volume with Large Dimensions</v>
       </c>
       <c r="F46" s="38" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
       <c r="G46" s="38" t="s">
         <v>1549</v>
@@ -13948,19 +13986,19 @@
         <v>1550</v>
       </c>
       <c r="J46" s="38" t="s">
-        <v>1692</v>
+        <v>1691</v>
       </c>
       <c r="K46" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="L46" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="M46" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="N46" s="38" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="S46">
         <v>1</v>
@@ -13971,7 +14009,7 @@
         <v>70</v>
       </c>
       <c r="B47" s="41" t="s">
-        <v>1693</v>
+        <v>1692</v>
       </c>
       <c r="C47" s="38" t="s">
         <v>69</v>
@@ -13981,12 +14019,12 @@
         <v>TRAVEL &gt; 4 MINS</v>
       </c>
       <c r="V47" s="38" t="s">
-        <v>1694</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="75" spans="1:14" ht="34">
       <c r="A75" s="197" t="s">
-        <v>1695</v>
+        <v>1694</v>
       </c>
       <c r="B75" s="197" t="s">
         <v>56</v>
@@ -14054,7 +14092,7 @@
         <v>1541</v>
       </c>
       <c r="I76" s="38" t="s">
-        <v>1696</v>
+        <v>1695</v>
       </c>
       <c r="J76" s="38" t="s">
         <v>1543</v>
@@ -14063,13 +14101,13 @@
         <v>1544</v>
       </c>
       <c r="L76" s="38" t="s">
+        <v>1696</v>
+      </c>
+      <c r="M76" s="38" t="s">
+        <v>1595</v>
+      </c>
+      <c r="N76" s="38" t="s">
         <v>1697</v>
-      </c>
-      <c r="M76" s="38" t="s">
-        <v>1596</v>
-      </c>
-      <c r="N76" s="38" t="s">
-        <v>1698</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="409.6">
@@ -14086,7 +14124,7 @@
         <v>144</v>
       </c>
       <c r="E77" s="38" t="s">
-        <v>1699</v>
+        <v>1698</v>
       </c>
       <c r="F77" s="38" t="s">
         <v>1549</v>
@@ -14098,10 +14136,10 @@
         <v>1550</v>
       </c>
       <c r="I77" s="38" t="s">
+        <v>1699</v>
+      </c>
+      <c r="J77" s="38" t="s">
         <v>1700</v>
-      </c>
-      <c r="J77" s="38" t="s">
-        <v>1701</v>
       </c>
       <c r="K77" s="38" t="s">
         <v>1544</v>
@@ -14110,15 +14148,15 @@
         <v>1556</v>
       </c>
       <c r="M77" s="38" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N77" s="38" t="s">
         <v>1702</v>
-      </c>
-      <c r="N77" s="38" t="s">
-        <v>1703</v>
       </c>
     </row>
     <row r="92" spans="1:19">
       <c r="A92" s="241" t="s">
-        <v>1704</v>
+        <v>1703</v>
       </c>
       <c r="B92" s="241"/>
     </row>
@@ -14133,19 +14171,19 @@
         <v>228</v>
       </c>
       <c r="D93" s="208" t="s">
+        <v>1704</v>
+      </c>
+      <c r="E93" s="208" t="s">
         <v>1705</v>
       </c>
-      <c r="E93" s="208" t="s">
+      <c r="F93" s="208" t="s">
         <v>1706</v>
       </c>
-      <c r="F93" s="208" t="s">
+      <c r="G93" s="209" t="s">
+        <v>1706</v>
+      </c>
+      <c r="H93" s="208" t="s">
         <v>1707</v>
-      </c>
-      <c r="G93" s="209" t="s">
-        <v>1707</v>
-      </c>
-      <c r="H93" s="208" t="s">
-        <v>1708</v>
       </c>
       <c r="I93" s="208" t="s">
         <v>1543</v>
@@ -14154,10 +14192,10 @@
         <v>1544</v>
       </c>
       <c r="K93" s="208" t="s">
+        <v>1708</v>
+      </c>
+      <c r="L93" s="208" t="s">
         <v>1709</v>
-      </c>
-      <c r="L93" s="208" t="s">
-        <v>1710</v>
       </c>
       <c r="M93" s="208">
         <v>1</v>
@@ -14170,7 +14208,7 @@
       <c r="Q93" s="208"/>
       <c r="R93" s="209"/>
       <c r="S93" s="208" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="94" spans="1:19" ht="409.6">
@@ -14184,19 +14222,19 @@
         <v>129</v>
       </c>
       <c r="D94" s="208" t="s">
+        <v>1710</v>
+      </c>
+      <c r="E94" s="208" t="s">
         <v>1711</v>
       </c>
-      <c r="E94" s="208" t="s">
+      <c r="F94" s="208" t="s">
+        <v>1706</v>
+      </c>
+      <c r="G94" s="209" t="s">
+        <v>1706</v>
+      </c>
+      <c r="H94" s="208" t="s">
         <v>1712</v>
-      </c>
-      <c r="F94" s="208" t="s">
-        <v>1707</v>
-      </c>
-      <c r="G94" s="209" t="s">
-        <v>1707</v>
-      </c>
-      <c r="H94" s="208" t="s">
-        <v>1713</v>
       </c>
       <c r="I94" s="208" t="s">
         <v>1543</v>
@@ -14205,10 +14243,10 @@
         <v>1544</v>
       </c>
       <c r="K94" s="208" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="L94" s="208" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="M94" s="208">
         <v>1</v>
@@ -14221,7 +14259,7 @@
       <c r="Q94" s="208"/>
       <c r="R94" s="209"/>
       <c r="S94" s="208" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="95" spans="1:19" ht="409.6">
@@ -14235,31 +14273,31 @@
         <v>175</v>
       </c>
       <c r="D95" s="208" t="s">
+        <v>1714</v>
+      </c>
+      <c r="E95" s="208" t="s">
         <v>1715</v>
       </c>
-      <c r="E95" s="208" t="s">
+      <c r="F95" s="208" t="s">
+        <v>1706</v>
+      </c>
+      <c r="G95" s="209" t="s">
+        <v>1706</v>
+      </c>
+      <c r="H95" s="208" t="s">
         <v>1716</v>
       </c>
-      <c r="F95" s="208" t="s">
-        <v>1707</v>
-      </c>
-      <c r="G95" s="209" t="s">
-        <v>1707</v>
-      </c>
-      <c r="H95" s="208" t="s">
+      <c r="I95" s="208" t="s">
         <v>1717</v>
-      </c>
-      <c r="I95" s="208" t="s">
-        <v>1718</v>
       </c>
       <c r="J95" s="208" t="s">
         <v>1544</v>
       </c>
       <c r="K95" s="208" t="s">
+        <v>1718</v>
+      </c>
+      <c r="L95" s="208" t="s">
         <v>1719</v>
-      </c>
-      <c r="L95" s="208" t="s">
-        <v>1720</v>
       </c>
       <c r="M95" s="208">
         <v>1</v>
@@ -14272,7 +14310,7 @@
       <c r="Q95" s="208"/>
       <c r="R95" s="209"/>
       <c r="S95" s="208" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="109" spans="1:14" ht="256">
@@ -14283,25 +14321,25 @@
         <v>69</v>
       </c>
       <c r="C109" s="38" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="D109" s="38" t="s">
         <v>172</v>
       </c>
       <c r="E109" s="38" t="s">
+        <v>1722</v>
+      </c>
+      <c r="F109" s="38" t="s">
         <v>1723</v>
-      </c>
-      <c r="F109" s="38" t="s">
-        <v>1724</v>
       </c>
       <c r="G109" s="38" t="s">
         <v>171</v>
       </c>
       <c r="H109" t="s">
+        <v>1724</v>
+      </c>
+      <c r="I109" s="38" t="s">
         <v>1725</v>
-      </c>
-      <c r="I109" s="38" t="s">
-        <v>1726</v>
       </c>
       <c r="K109" s="38" t="s">
         <v>1544</v>
@@ -14310,10 +14348,10 @@
         <v>1556</v>
       </c>
       <c r="M109" s="38" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="N109" s="38" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
     </row>
   </sheetData>
@@ -14356,13 +14394,13 @@
         <v>229</v>
       </c>
       <c r="B1" t="s">
+        <v>1727</v>
+      </c>
+      <c r="C1" s="38" t="s">
         <v>1728</v>
       </c>
-      <c r="C1" s="38" t="s">
+      <c r="D1" s="38" t="s">
         <v>1729</v>
-      </c>
-      <c r="D1" s="38" t="s">
-        <v>1730</v>
       </c>
       <c r="E1" s="38" t="s">
         <v>1534</v>
@@ -14383,13 +14421,13 @@
         <v>28</v>
       </c>
       <c r="K1" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="L1" t="s">
         <v>246</v>
       </c>
       <c r="M1" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="N1" t="s">
         <v>245</v>
@@ -14403,13 +14441,13 @@
         <v>76</v>
       </c>
       <c r="C2" s="38" t="s">
+        <v>1732</v>
+      </c>
+      <c r="D2" t="s">
         <v>1733</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>1734</v>
-      </c>
-      <c r="E2" t="s">
-        <v>1735</v>
       </c>
       <c r="F2" s="38" t="s">
         <v>1543</v>
@@ -14421,10 +14459,10 @@
         <v>1556</v>
       </c>
       <c r="I2" s="38" t="s">
+        <v>1735</v>
+      </c>
+      <c r="J2" s="41" t="s">
         <v>1736</v>
-      </c>
-      <c r="J2" s="41" t="s">
-        <v>1737</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -14445,13 +14483,13 @@
         <v>ALPHA OPEN ADJUSTMENTS &gt; 35DAYS</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="D3" s="195" t="s">
+        <v>1737</v>
+      </c>
+      <c r="E3" s="196" t="s">
         <v>1738</v>
-      </c>
-      <c r="E3" s="196" t="s">
-        <v>1739</v>
       </c>
       <c r="F3" s="38" t="s">
         <v>1543</v>
@@ -14460,10 +14498,10 @@
         <v>1544</v>
       </c>
       <c r="H3" s="38" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="I3" s="38" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="L3">
         <v>1</v>
@@ -14483,13 +14521,13 @@
         <v>210</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
       <c r="D4" t="s">
+        <v>1740</v>
+      </c>
+      <c r="E4" s="38" t="s">
         <v>1741</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>1742</v>
       </c>
       <c r="F4" s="38" t="s">
         <v>1543</v>
@@ -14498,13 +14536,13 @@
         <v>1544</v>
       </c>
       <c r="H4" s="38" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="I4" s="38" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="J4" s="38" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -14524,28 +14562,28 @@
         <v>88</v>
       </c>
       <c r="C5" s="38" t="s">
+        <v>1743</v>
+      </c>
+      <c r="D5" s="38" t="s">
         <v>1744</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="E5" s="38" t="s">
         <v>1745</v>
       </c>
-      <c r="E5" s="38" t="s">
+      <c r="F5" s="38" t="s">
         <v>1746</v>
-      </c>
-      <c r="F5" s="38" t="s">
-        <v>1747</v>
       </c>
       <c r="G5" s="38" t="s">
         <v>1544</v>
       </c>
       <c r="H5" s="38" t="s">
+        <v>1747</v>
+      </c>
+      <c r="I5" s="38" t="s">
         <v>1748</v>
       </c>
-      <c r="I5" s="38" t="s">
+      <c r="J5" s="41" t="s">
         <v>1749</v>
-      </c>
-      <c r="J5" s="41" t="s">
-        <v>1750</v>
       </c>
       <c r="L5" s="38">
         <v>1</v>
@@ -14565,28 +14603,28 @@
         <v>86</v>
       </c>
       <c r="C6" s="38" t="s">
+        <v>1750</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1733</v>
+      </c>
+      <c r="E6" s="199" t="s">
         <v>1751</v>
       </c>
-      <c r="D6" t="s">
-        <v>1734</v>
-      </c>
-      <c r="E6" s="199" t="s">
+      <c r="F6" s="38" t="s">
         <v>1752</v>
-      </c>
-      <c r="F6" s="38" t="s">
-        <v>1753</v>
       </c>
       <c r="G6" t="s">
         <v>1544</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="I6" s="38" t="s">
+        <v>1753</v>
+      </c>
+      <c r="J6" s="41" t="s">
         <v>1754</v>
-      </c>
-      <c r="J6" s="41" t="s">
-        <v>1755</v>
       </c>
       <c r="L6">
         <v>1</v>
@@ -14607,16 +14645,16 @@
         <v>ASW ASN ERROR</v>
       </c>
       <c r="C7" s="38" t="s">
+        <v>1755</v>
+      </c>
+      <c r="D7" t="s">
         <v>1756</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>1757</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" s="38" t="s">
         <v>1758</v>
-      </c>
-      <c r="F7" s="38" t="s">
-        <v>1759</v>
       </c>
       <c r="G7" t="s">
         <v>1544</v>
@@ -14625,10 +14663,10 @@
         <v>1556</v>
       </c>
       <c r="I7" s="38" t="s">
+        <v>1759</v>
+      </c>
+      <c r="J7" s="210" t="s">
         <v>1760</v>
-      </c>
-      <c r="J7" s="210" t="s">
-        <v>1761</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -14648,16 +14686,16 @@
         <v>138</v>
       </c>
       <c r="C8" s="38" t="s">
+        <v>1761</v>
+      </c>
+      <c r="D8" t="s">
         <v>1762</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="38" t="s">
         <v>1763</v>
       </c>
-      <c r="E8" s="38" t="s">
+      <c r="F8" t="s">
         <v>1764</v>
-      </c>
-      <c r="F8" t="s">
-        <v>1765</v>
       </c>
       <c r="G8" t="s">
         <v>1544</v>
@@ -14666,10 +14704,10 @@
         <v>1556</v>
       </c>
       <c r="I8" s="38" t="s">
+        <v>1765</v>
+      </c>
+      <c r="J8" s="41" t="s">
         <v>1766</v>
-      </c>
-      <c r="J8" s="41" t="s">
-        <v>1767</v>
       </c>
       <c r="K8">
         <v>1</v>
@@ -14689,13 +14727,13 @@
         <v>146</v>
       </c>
       <c r="C9" s="38" t="s">
+        <v>1767</v>
+      </c>
+      <c r="D9" t="s">
         <v>1768</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" s="199" t="s">
         <v>1769</v>
-      </c>
-      <c r="E9" s="199" t="s">
-        <v>1770</v>
       </c>
       <c r="F9" s="38" t="s">
         <v>1543</v>
@@ -14704,13 +14742,13 @@
         <v>1544</v>
       </c>
       <c r="H9" s="38" t="s">
+        <v>1770</v>
+      </c>
+      <c r="I9" s="38" t="s">
         <v>1771</v>
       </c>
-      <c r="I9" s="38" t="s">
+      <c r="J9" s="38" t="s">
         <v>1772</v>
-      </c>
-      <c r="J9" s="38" t="s">
-        <v>1773</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -14730,13 +14768,13 @@
         <v>207</v>
       </c>
       <c r="C10" s="38" t="s">
+        <v>1773</v>
+      </c>
+      <c r="D10" t="s">
         <v>1774</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" s="38" t="s">
         <v>1775</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>1776</v>
       </c>
       <c r="F10" s="38" t="s">
         <v>1543</v>
@@ -14748,10 +14786,10 @@
         <v>1556</v>
       </c>
       <c r="I10" s="38" t="s">
+        <v>1776</v>
+      </c>
+      <c r="J10" s="41" t="s">
         <v>1777</v>
-      </c>
-      <c r="J10" s="41" t="s">
-        <v>1778</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -14770,7 +14808,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="203" t="s">
-        <v>1779</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15" customHeight="1">
@@ -14879,39 +14917,39 @@
   <sheetData>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>1779</v>
+      </c>
+      <c r="B2" t="s">
         <v>1780</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1781</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
+        <v>1781</v>
+      </c>
+      <c r="B3" t="s">
         <v>1782</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1783</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
+        <v>1784</v>
+      </c>
+      <c r="B6" t="s">
         <v>1785</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1786</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
+        <v>1786</v>
+      </c>
+      <c r="B7" t="s">
         <v>1787</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1788</v>
       </c>
     </row>
   </sheetData>
@@ -14934,16 +14972,16 @@
         <v>46070</v>
       </c>
       <c r="C4" t="s">
+        <v>1788</v>
+      </c>
+      <c r="D4" t="s">
         <v>1789</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>1790</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>1791</v>
-      </c>
-      <c r="F4" t="s">
-        <v>1792</v>
       </c>
     </row>
   </sheetData>
@@ -14965,20 +15003,20 @@
   <sheetData>
     <row r="10" spans="4:8" ht="16" thickBot="1"/>
     <row r="11" spans="4:8">
-      <c r="D11" s="216" t="s">
+      <c r="D11" s="229" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="217"/>
-      <c r="F11" s="217"/>
-      <c r="G11" s="217"/>
-      <c r="H11" s="218"/>
+      <c r="E11" s="230"/>
+      <c r="F11" s="230"/>
+      <c r="G11" s="230"/>
+      <c r="H11" s="231"/>
     </row>
     <row r="12" spans="4:8" ht="16" thickBot="1">
-      <c r="D12" s="219"/>
-      <c r="E12" s="220"/>
-      <c r="F12" s="220"/>
-      <c r="G12" s="220"/>
-      <c r="H12" s="221"/>
+      <c r="D12" s="232"/>
+      <c r="E12" s="233"/>
+      <c r="F12" s="233"/>
+      <c r="G12" s="233"/>
+      <c r="H12" s="234"/>
     </row>
     <row r="13" spans="4:8" ht="17" thickBot="1">
       <c r="D13" s="145" t="s">
@@ -46173,6 +46211,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005977094627AF1147A308E96CD6855572" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="385c3e00234168da4d1aac2c9e9aca32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4b65c1a-daac-4fd9-ba72-b6c84fe15ed4" xmlns:ns3="bda85dd2-6cbf-49e9-8f64-78faf376eb43" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="16a5d8217ce5de02597adbdd380d4920" ns2:_="" ns3:_="">
     <xsd:import namespace="f4b65c1a-daac-4fd9-ba72-b6c84fe15ed4"/>
@@ -46413,15 +46460,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -46434,6 +46472,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E688908-2AF4-423A-99D9-C040C1537B7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BC6226C-693E-49EB-9F6E-2AD1482C940B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -46452,14 +46498,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E688908-2AF4-423A-99D9-C040C1537B7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A314CBA-DDFC-407B-913E-456EF7A72CB2}">
   <ds:schemaRefs>

</xml_diff>